<commit_message>
add overtimes to workflow
</commit_message>
<xml_diff>
--- a/assets/ods/global_revenue_template.xlsx
+++ b/assets/ods/global_revenue_template.xlsx
@@ -13,27 +13,27 @@
     <sheet name="Feuil3" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="CONTRIBUTION_DIFFUSEUR_AGESSA" vbProcedure="false">Feuil1!$C$15</definedName>
-    <definedName function="false" hidden="false" name="CONTRIBUTION_RETRAITE" vbProcedure="false">Feuil1!$C$14</definedName>
-    <definedName function="false" hidden="false" name="DIFFERENCE_RECETTE_MINIMUM_GARANTI" vbProcedure="false">Feuil1!$G$13</definedName>
-    <definedName function="false" hidden="false" name="DROIT_D_AUTEUR" vbProcedure="false">Feuil1!$C$13</definedName>
+    <definedName function="false" hidden="false" name="CONTRIBUTION_DIFFUSEUR_AGESSA" vbProcedure="false">Feuil1!$C$16</definedName>
+    <definedName function="false" hidden="false" name="CONTRIBUTION_RETRAITE" vbProcedure="false">Feuil1!$C$15</definedName>
+    <definedName function="false" hidden="false" name="DIFFERENCE_RECETTE_MINIMUM_GARANTI" vbProcedure="false">Feuil1!$G$14</definedName>
+    <definedName function="false" hidden="false" name="DROIT_D_AUTEUR" vbProcedure="false">Feuil1!$C$14</definedName>
     <definedName function="false" hidden="false" name="GRATUIT" vbProcedure="false">Feuil1!$F1</definedName>
     <definedName function="false" hidden="false" name="LIGNE_APPLICABLE" vbProcedure="false">Feuil1!$B1</definedName>
-    <definedName function="false" hidden="false" name="MINIMUM_COMPAGNIE_PAR_REPRESENTATION" vbProcedure="false">Feuil1!$G$12</definedName>
-    <definedName function="false" hidden="false" name="MINIMUM_GARANTI_THEATRE_PAR_REPRESENTATION" vbProcedure="false">Feuil1!$G$10</definedName>
-    <definedName function="false" hidden="false" name="MINIMUM_GARANTI_TOTAL" vbProcedure="false">Feuil1!$G$11</definedName>
+    <definedName function="false" hidden="false" name="MINIMUM_COMPAGNIE_PAR_REPRESENTATION" vbProcedure="false">Feuil1!$G$13</definedName>
+    <definedName function="false" hidden="false" name="MINIMUM_GARANTI_THEATRE_PAR_REPRESENTATION" vbProcedure="false">Feuil1!$G$11</definedName>
+    <definedName function="false" hidden="false" name="MINIMUM_GARANTI_TOTAL" vbProcedure="false">Feuil1!$G$12</definedName>
     <definedName function="false" hidden="false" name="NOMBRE_REPRESENTATIONS" vbProcedure="false">Feuil1!$A$9:$A$9</definedName>
-    <definedName function="false" hidden="false" name="PART_COMPAGNIE" vbProcedure="false">Feuil1!$F$16</definedName>
-    <definedName function="false" hidden="false" name="PART_THEATRE" vbProcedure="false">Feuil1!$F$15</definedName>
+    <definedName function="false" hidden="false" name="PART_COMPAGNIE" vbProcedure="false">Feuil1!$F$17</definedName>
+    <definedName function="false" hidden="false" name="PART_THEATRE" vbProcedure="false">Feuil1!$F$16</definedName>
     <definedName function="false" hidden="false" name="PAYANT" vbProcedure="false">Feuil1!$E1</definedName>
     <definedName function="false" hidden="false" name="RECETTES" vbProcedure="false">Feuil1!$C$9:$C$9</definedName>
-    <definedName function="false" hidden="false" name="RECETTE_BRUTE" vbProcedure="false">Feuil1!$C$10</definedName>
-    <definedName function="false" hidden="false" name="RECETTE_HTVA" vbProcedure="false">Feuil1!$C$12</definedName>
-    <definedName function="false" hidden="false" name="RECETTE_NETTE" vbProcedure="false">Feuil1!$C$17</definedName>
-    <definedName function="false" hidden="false" name="TAXE_PARAFISCALE" vbProcedure="false">Feuil1!$C$16</definedName>
-    <definedName function="false" hidden="false" name="TOTAL_THEATRE" vbProcedure="false">Feuil1!$G$15</definedName>
-    <definedName function="false" hidden="false" name="TVA" vbProcedure="false">Feuil1!$C$11</definedName>
-    <definedName function="false" hidden="false" name="TVA_DIFFERENCE_MINIMUM_GARANTI" vbProcedure="false">Feuil1!$G$14</definedName>
+    <definedName function="false" hidden="false" name="RECETTE_BRUTE" vbProcedure="false">Feuil1!$C$11</definedName>
+    <definedName function="false" hidden="false" name="RECETTE_HTVA" vbProcedure="false">Feuil1!$C$13</definedName>
+    <definedName function="false" hidden="false" name="RECETTE_NETTE" vbProcedure="false">Feuil1!$C$18</definedName>
+    <definedName function="false" hidden="false" name="TAXE_PARAFISCALE" vbProcedure="false">Feuil1!$C$17</definedName>
+    <definedName function="false" hidden="false" name="TOTAL_THEATRE" vbProcedure="false">Feuil1!$G$16</definedName>
+    <definedName function="false" hidden="false" name="TVA" vbProcedure="false">Feuil1!$C$12</definedName>
+    <definedName function="false" hidden="false" name="TVA_DIFFERENCE_MINIMUM_GARANTI" vbProcedure="false">Feuil1!$G$15</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="40">
   <si>
     <t xml:space="preserve">BORDEREAU DE RECETTE :</t>
   </si>
@@ -80,31 +80,28 @@
     <t xml:space="preserve">NOMBRE DE</t>
   </si>
   <si>
+    <t xml:space="preserve">DATE</t>
+  </si>
+  <si>
     <t xml:space="preserve">RECETTE</t>
   </si>
   <si>
     <t xml:space="preserve">NOMBRE</t>
   </si>
   <si>
+    <t xml:space="preserve">PAYANT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRATUIT</t>
+  </si>
+  <si>
     <t xml:space="preserve">REPRESENT.</t>
   </si>
   <si>
-    <t xml:space="preserve">DATE</t>
-  </si>
-  <si>
     <t xml:space="preserve">BRUTE</t>
   </si>
   <si>
     <t xml:space="preserve">D'ENTREES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PAYANT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRATUIT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
     <t xml:space="preserve">RECETTE BRUTE :</t>
@@ -189,7 +186,7 @@
     <numFmt numFmtId="175" formatCode="\ * #,##0.00\ [$€-81D]\ ;\-* #,##0.00\ [$€-81D]\ ;\ * \-#\ [$€-81D]\ ;\ @\ "/>
     <numFmt numFmtId="176" formatCode="\ * #,##0.00\ [$€-1]\ ;\-* #,##0.00\ [$€-1]\ ;\ * \-#\ [$€-1]\ ;\ @\ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -263,8 +260,8 @@
       <b val="true"/>
       <sz val="12"/>
       <color rgb="FF003366"/>
-      <name val="TimesNewRomanPS"/>
-      <family val="0"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="1"/>
     </font>
     <font>
@@ -315,19 +312,25 @@
       <b val="true"/>
       <sz val="12"/>
       <color rgb="FF003366"/>
+      <name val="TimesNewRomanPS"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
+      <name val="MS Sans Serif"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="TimesNewRomanPS"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="MS Sans Serif"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -352,7 +355,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="7">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -378,7 +381,7 @@
       <left style="thin"/>
       <right/>
       <top style="thin"/>
-      <bottom/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -386,20 +389,6 @@
       <right style="thin"/>
       <top/>
       <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -414,27 +403,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -466,7 +434,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="56">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -524,7 +492,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -532,15 +500,11 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -571,63 +535,55 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -635,23 +591,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="173" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="18" fillId="0" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="174" fontId="11" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -659,35 +611,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -695,10 +623,6 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -711,11 +635,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -725,6 +649,14 @@
     </xf>
     <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -851,7 +783,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="11.171875" defaultRowHeight="14.65" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="45.7"/>
@@ -946,303 +878,340 @@
       <c r="A7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="14"/>
+      <c r="B7" s="14" t="s">
+        <v>11</v>
+      </c>
       <c r="C7" s="15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="16"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="18"/>
+        <v>13</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="0"/>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="19" t="s">
+      <c r="A8" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="B8" s="14"/>
+      <c r="C8" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="D8" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="19" t="s">
-        <v>19</v>
-      </c>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="0"/>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="21" t="n">
         <v>45701</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="22" t="n">
         <v>520</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="23" t="n">
         <f aca="false">PAYANT + GRATUIT</f>
         <v>27</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="23" t="n">
         <v>25</v>
       </c>
-      <c r="F9" s="25" t="n">
+      <c r="F9" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="21"/>
+      <c r="G9" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="27"/>
-      <c r="C10" s="28" t="n">
+      <c r="A10" s="0"/>
+      <c r="B10" s="0"/>
+      <c r="C10" s="0"/>
+      <c r="D10" s="0"/>
+      <c r="E10" s="0"/>
+      <c r="F10" s="0"/>
+      <c r="G10" s="0"/>
+    </row>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="26"/>
+      <c r="C11" s="27" t="n">
         <f aca="false">SUM(RECETTES)</f>
         <v>520</v>
       </c>
-      <c r="D10" s="29"/>
-      <c r="E10" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="31"/>
-      <c r="G10" s="32" t="n">
+      <c r="D11" s="28"/>
+      <c r="E11" s="29" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="30"/>
+      <c r="G11" s="31" t="n">
         <f aca="false">100</f>
         <v>100</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="33" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="34"/>
-      <c r="C11" s="35" t="n">
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="26"/>
+      <c r="C12" s="27" t="n">
         <f aca="false">(RECETTE_BRUTE-RECETTE_HTVA)</f>
         <v>10.6953966699314</v>
       </c>
-      <c r="D11" s="36"/>
-      <c r="E11" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="37"/>
-      <c r="G11" s="32" t="n">
+      <c r="D12" s="33"/>
+      <c r="E12" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="34"/>
+      <c r="G12" s="31" t="n">
         <f aca="false">MINIMUM_GARANTI_THEATRE_PAR_REPRESENTATION*SUM(NOMBRE_REPRESENTATIONS)</f>
         <v>100</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="34"/>
-      <c r="C12" s="35" t="n">
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="26"/>
+      <c r="C13" s="27" t="n">
         <f aca="false">(RECETTE_BRUTE/1.021)</f>
         <v>509.304603330069</v>
       </c>
-      <c r="D12" s="36"/>
-      <c r="E12" s="30" t="s">
+      <c r="D13" s="33"/>
+      <c r="E13" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" s="34"/>
+      <c r="G13" s="31" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="F12" s="37"/>
-      <c r="G12" s="32" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="33" t="s">
+      <c r="B14" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="35" t="n">
+      <c r="C14" s="27" t="n">
         <f aca="false">IF(LIGNE_APPLICABLE="Applicable",RECETTE_HTVA*0.12,0)</f>
         <v>61.1165523996082</v>
       </c>
-      <c r="D13" s="36"/>
-      <c r="E13" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="F13" s="37"/>
-      <c r="G13" s="32" t="n">
+      <c r="D14" s="33"/>
+      <c r="E14" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="34"/>
+      <c r="G14" s="31" t="n">
         <f aca="false">-MIN(RECETTE_NETTE - MINIMUM_GARANTI_TOTAL , 0)</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="33" t="s">
-        <v>29</v>
-      </c>
-      <c r="B14" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="35" t="n">
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="27" t="n">
         <f aca="false">IF(LIGNE_APPLICABLE="Applicable",RECETTE_HTVA*0.01,0)</f>
         <v>5.09304603330069</v>
       </c>
-      <c r="D14" s="36"/>
-      <c r="E14" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="F14" s="37"/>
-      <c r="G14" s="32" t="n">
+      <c r="D15" s="33"/>
+      <c r="E15" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="34"/>
+      <c r="G15" s="31" t="n">
         <f aca="false">0.2 * DIFFERENCE_RECETTE_MINIMUM_GARANTI</f>
         <v>-0</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="33" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="35" t="n">
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="27" t="n">
         <f aca="false">IF(LIGNE_APPLICABLE="Applicable",DROIT_D_AUTEUR * 0.01,0)</f>
         <v>0.611165523996082</v>
       </c>
-      <c r="D15" s="36"/>
-      <c r="E15" s="41" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" s="42" t="n">
+      <c r="D16" s="33"/>
+      <c r="E16" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" s="39" t="n">
         <v>0.5</v>
       </c>
-      <c r="G15" s="43" t="n">
+      <c r="G16" s="40" t="n">
         <f aca="false">MINIMUM_GARANTI_TOTAL + TVA_DIFFERENCE_MINIMUM_GARANTI + (RECETTE_NETTE - MIN(RECETTE_NETTE - MINIMUM_GARANTI_TOTAL, SUM(NOMBRE_REPRESENTATIONS) * MINIMUM_COMPAGNIE_PAR_REPRESENTATION)-MINIMUM_GARANTI_TOTAL) * PART_THEATRE</f>
         <v>212.329089128306</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="33" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="44"/>
-      <c r="C16" s="35" t="n">
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="28"/>
+      <c r="C17" s="27" t="n">
         <f aca="false">(RECETTE_HTVA*0.035)</f>
         <v>17.8256611165524</v>
       </c>
-      <c r="D16" s="36"/>
-      <c r="E16" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="F16" s="42" t="n">
+      <c r="D17" s="33"/>
+      <c r="E17" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="F17" s="39" t="n">
         <v>0.5</v>
       </c>
-      <c r="G16" s="46" t="n">
+      <c r="G17" s="42" t="n">
         <f aca="false">RECETTE_NETTE - TOTAL_THEATRE</f>
         <v>212.329089128306</v>
       </c>
-      <c r="I16" s="47"/>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="48" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17" s="49"/>
-      <c r="C17" s="50" t="n">
+      <c r="I17" s="43"/>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="28"/>
+      <c r="C18" s="44" t="n">
         <f aca="false">RECETTE_BRUTE - TVA-DROIT_D_AUTEUR - CONTRIBUTION_RETRAITE - CONTRIBUTION_DIFFUSEUR_AGESSA - TAXE_PARAFISCALE</f>
         <v>424.658178256611</v>
       </c>
-      <c r="D17" s="51"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="53"/>
-      <c r="G17" s="53"/>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="54"/>
-      <c r="B18" s="55"/>
-      <c r="C18" s="56"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="58"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-    </row>
-    <row r="19" s="63" customFormat="true" ht="41" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="59" t="s">
+      <c r="D18" s="30"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="45"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="33"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+    </row>
+    <row r="22" s="52" customFormat="true" ht="41" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="48" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" s="49"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="51"/>
+      <c r="E22" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="60"/>
-      <c r="C19" s="61"/>
-      <c r="D19" s="62"/>
-      <c r="E19" s="59" t="s">
+    </row>
+    <row r="23" s="52" customFormat="true" ht="38.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="53" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="20" s="63" customFormat="true" ht="38.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="64" t="s">
+      <c r="B23" s="54" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="64" t="s">
+      <c r="C23" s="50"/>
+      <c r="D23" s="54"/>
+      <c r="E23" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="61"/>
-      <c r="D20" s="64"/>
-      <c r="E20" s="59" t="s">
-        <v>40</v>
-      </c>
-      <c r="F20" s="59" t="s">
-        <v>39</v>
-      </c>
-      <c r="G20" s="64"/>
-    </row>
-    <row r="21" s="63" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="64"/>
-      <c r="B21" s="64"/>
-      <c r="C21" s="61"/>
-      <c r="D21" s="64"/>
-      <c r="E21" s="64"/>
-      <c r="F21" s="64"/>
-      <c r="G21" s="64"/>
-    </row>
-    <row r="22" s="63" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="64"/>
-      <c r="G22" s="64"/>
-    </row>
-    <row r="23" s="63" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="64"/>
-      <c r="G23" s="64"/>
-    </row>
-    <row r="24" s="63" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="64"/>
-      <c r="G24" s="64"/>
-    </row>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="26" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="27" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="F23" s="55" t="s">
+        <v>38</v>
+      </c>
+      <c r="G23" s="54"/>
+    </row>
+    <row r="24" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="54"/>
+      <c r="B24" s="54"/>
+      <c r="C24" s="50"/>
+      <c r="D24" s="54"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="54"/>
+      <c r="G24" s="54"/>
+    </row>
+    <row r="25" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="54"/>
+    </row>
+    <row r="26" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="54"/>
+    </row>
+    <row r="27" s="52" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="54"/>
+      <c r="G27" s="54"/>
+    </row>
+    <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="29" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="31" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="32" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="33" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="34" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G7:G8"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>